<commit_message>
Improve metadata extraction and finalize error handling
</commit_message>
<xml_diff>
--- a/output/dicom_metadata.xlsx
+++ b/output/dicom_metadata.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,6 +442,36 @@
           <t>Manufacturer</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Institution Name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Study Description</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Series Description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Body Part Examined</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Rows</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Columns</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -467,6 +497,36 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>GE MEDICAL SYSTEMS</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>JFK IMAGING CENTER</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>e+1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Not Available</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>128</t>
         </is>
       </c>
     </row>

</xml_diff>